<commit_message>
Improvement: Refined fuzzy rules and added sorting tie-breaker (score > service > price)
</commit_message>
<xml_diff>
--- a/Kode/Python/ranking.xlsx
+++ b/Kode/Python/ranking.xlsx
@@ -440,13 +440,13 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>25</v>
+        <v>79</v>
       </c>
       <c r="B2" t="n">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C2" t="n">
-        <v>34513</v>
+        <v>22360</v>
       </c>
       <c r="D2" t="n">
         <v>100</v>
@@ -454,13 +454,13 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>15</v>
+        <v>80</v>
       </c>
       <c r="B3" t="n">
-        <v>55</v>
+        <v>89</v>
       </c>
       <c r="C3" t="n">
-        <v>22346</v>
+        <v>22012</v>
       </c>
       <c r="D3" t="n">
         <v>100</v>
@@ -468,13 +468,13 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>22</v>
+        <v>78</v>
       </c>
       <c r="B4" t="n">
-        <v>99</v>
+        <v>86</v>
       </c>
       <c r="C4" t="n">
-        <v>39211</v>
+        <v>27315</v>
       </c>
       <c r="D4" t="n">
         <v>100</v>
@@ -482,13 +482,13 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>23</v>
+        <v>69</v>
       </c>
       <c r="B5" t="n">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="C5" t="n">
-        <v>22825</v>
+        <v>24551</v>
       </c>
       <c r="D5" t="n">
         <v>100</v>
@@ -496,13 +496,13 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>27</v>
+        <v>86</v>
       </c>
       <c r="B6" t="n">
-        <v>53</v>
+        <v>84</v>
       </c>
       <c r="C6" t="n">
-        <v>23319</v>
+        <v>29811</v>
       </c>
       <c r="D6" t="n">
         <v>100</v>

</xml_diff>

<commit_message>
Enhancement: Added 'Kesimpulan' column to ranking and generated premium visualizations (V2)
</commit_message>
<xml_diff>
--- a/Kode/Python/ranking.xlsx
+++ b/Kode/Python/ranking.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -437,6 +437,11 @@
           <t>Skor Kelayakan</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Kesimpulan</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -451,6 +456,11 @@
       <c r="D2" t="n">
         <v>100</v>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Sangat Layak (Pilihan Utama)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -465,6 +475,11 @@
       <c r="D3" t="n">
         <v>100</v>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Sangat Layak (Pilihan Utama)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -479,6 +494,11 @@
       <c r="D4" t="n">
         <v>100</v>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Sangat Layak (Pilihan Utama)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -493,6 +513,11 @@
       <c r="D5" t="n">
         <v>100</v>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Sangat Layak (Pilihan Utama)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -506,6 +531,11 @@
       </c>
       <c r="D6" t="n">
         <v>100</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Sangat Layak (Pilihan Utama)</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>